<commit_message>
Itemize 2nd-floor duct demolition in contractor proposal
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MXDAyRkZCZe1vQqjdWh53W
</commit_message>
<xml_diff>
--- a/out/КП_Реновель_предложение_Подрядчика_v2.xlsx
+++ b/out/КП_Реновель_предложение_Подрядчика_v2.xlsx
@@ -288,7 +288,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="49">
+  <borders count="52">
     <border>
       <left/>
       <right/>
@@ -915,13 +915,46 @@
         <color rgb="00A6A6A6"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00A6A6A6"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00A6A6A6"/>
+      </right>
+      <top style="thin">
+        <color rgb="00A6A6A6"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00A6A6A6"/>
+      </right>
+      <top style="thin">
+        <color rgb="00A6A6A6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00A6A6A6"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="13" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="202">
+  <cellXfs count="209">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -1500,6 +1533,23 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="48" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="20" fillId="16" borderId="48" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="48" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="48" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="21" fillId="0" borderId="48" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="168" fontId="20" fillId="0" borderId="48" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -1903,7 +1953,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z349"/>
+  <dimension ref="A1:Z372"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.33203125" customWidth="1" style="20" min="1" max="1"/>
@@ -1914,7 +1964,7 @@
     <col width="16.6640625" customWidth="1" style="160" min="10" max="10"/>
     <col width="22.83203125" customWidth="1" style="161" min="11" max="11"/>
     <col width="22.5" customWidth="1" style="162" min="12" max="12"/>
-    <col hidden="1" style="155" min="13" max="13"/>
+    <col hidden="1" width="13" customWidth="1" style="155" min="13" max="13"/>
     <col width="19.1640625" bestFit="1" customWidth="1" style="155" min="15" max="15"/>
     <col width="13.5" bestFit="1" customWidth="1" style="155" min="16" max="16"/>
     <col width="18" customWidth="1" style="155" min="17" max="17"/>
@@ -23980,12 +24030,12 @@
       <c r="U335" s="196" t="n"/>
       <c r="V335" s="190" t="inlineStr">
         <is>
-          <t>Отдельное допсоглашение</t>
+          <t>Расписано по позициям</t>
         </is>
       </c>
       <c r="W335" s="190" t="inlineStr">
         <is>
-          <t>По Вашему замечанию распишем по позициям и оформим отдельным допсоглашением.</t>
+          <t>Расписано по Вашей просьбе ниже, строки 350-371 (объёмы по ведомости демонтажа). Включено в итог.</t>
         </is>
       </c>
       <c r="X335" s="174" t="inlineStr">
@@ -24208,6 +24258,7 @@
           <t>Итого по Вашему варианту (с учётом "ок")</t>
         </is>
       </c>
+      <c r="T342" s="202" t="n"/>
       <c r="U342" s="198">
         <f>SUM(Y5:Y327)</f>
         <v/>
@@ -24220,11 +24271,12 @@
     <row r="343" ht="28" customHeight="1" s="155">
       <c r="S343" s="197" t="inlineStr">
         <is>
-          <t>Итого по предложению Подрядчика</t>
-        </is>
-      </c>
+          <t>Итого по предложению Подрядчика (с расписанным демонтажом п. 6.71)</t>
+        </is>
+      </c>
+      <c r="T343" s="202" t="n"/>
       <c r="U343" s="198">
-        <f>SUM(Z5:Z327)</f>
+        <f>SUM(Z5:Z327)+L372</f>
         <v/>
       </c>
       <c r="V343" s="180" t="n"/>
@@ -24238,6 +24290,7 @@
           <t>Разница</t>
         </is>
       </c>
+      <c r="T344" s="202" t="n"/>
       <c r="U344" s="198">
         <f>U343-U342</f>
         <v/>
@@ -24247,22 +24300,30 @@
       <c r="Y344" s="180" t="n"/>
       <c r="Z344" s="180" t="n"/>
     </row>
-    <row r="345" ht="28" customHeight="1" s="155">
+    <row r="345" ht="42" customHeight="1" s="155">
       <c r="S345" s="197" t="inlineStr">
         <is>
-          <t>Дымоудаление и демонтажи - отдельным КП / допсоглашением, в итог не входят</t>
-        </is>
-      </c>
+          <t>Дымоудаление, демонтаж холодоснабжения и дренажа (7.9, 7.10), дренаж и подключение фанкойлов (5.35, 7.2, 7.8) - отдельным КП / допсоглашением, в итог не входят</t>
+        </is>
+      </c>
+      <c r="T345" s="202" t="n"/>
       <c r="U345" s="199" t="n"/>
       <c r="V345" s="180" t="n"/>
       <c r="W345" s="180" t="n"/>
       <c r="Y345" s="180" t="n"/>
       <c r="Z345" s="180" t="n"/>
     </row>
-    <row r="346" ht="27.95" customHeight="1" s="155">
-      <c r="S346" s="200" t="n"/>
-      <c r="T346" s="180" t="n"/>
-      <c r="U346" s="199" t="n"/>
+    <row r="346" ht="28" customHeight="1" s="155">
+      <c r="S346" s="203" t="inlineStr">
+        <is>
+          <t>в т.ч. демонтаж воздуховодов 2 эт. (п. 6.71), расписан ниже</t>
+        </is>
+      </c>
+      <c r="T346" s="202" t="n"/>
+      <c r="U346" s="204">
+        <f>L372</f>
+        <v/>
+      </c>
       <c r="V346" s="180" t="n"/>
       <c r="W346" s="180" t="n"/>
       <c r="Y346" s="180" t="n"/>
@@ -24278,6 +24339,11 @@
       <c r="Z347" s="180" t="n"/>
     </row>
     <row r="348">
+      <c r="A348" s="158" t="inlineStr">
+        <is>
+          <t>П. 6.71 ДЕМОНТАЖ ВОЗДУХОВОДОВ 2 ЭТАЖА - РАСПИСАНО ПО ПОЗИЦИЯМ (объёмы по ведомости демонтированного оборудования)</t>
+        </is>
+      </c>
       <c r="S348" s="180" t="n"/>
       <c r="T348" s="180" t="n"/>
       <c r="U348" s="180" t="n"/>
@@ -24287,6 +24353,36 @@
       <c r="Z348" s="180" t="n"/>
     </row>
     <row r="349" ht="80.09999999999999" customHeight="1" s="155">
+      <c r="A349" s="193" t="inlineStr">
+        <is>
+          <t>№ п/п</t>
+        </is>
+      </c>
+      <c r="B349" s="193" t="inlineStr">
+        <is>
+          <t>НАИМЕНОВАНИЕ</t>
+        </is>
+      </c>
+      <c r="C349" s="193" t="inlineStr">
+        <is>
+          <t>Ед. изм</t>
+        </is>
+      </c>
+      <c r="J349" s="193" t="inlineStr">
+        <is>
+          <t>Кол-во</t>
+        </is>
+      </c>
+      <c r="K349" s="193" t="inlineStr">
+        <is>
+          <t>Цена за ед., руб.</t>
+        </is>
+      </c>
+      <c r="L349" s="193" t="inlineStr">
+        <is>
+          <t>Всего, руб.</t>
+        </is>
+      </c>
       <c r="S349" s="200" t="n"/>
       <c r="T349" s="180" t="n"/>
       <c r="U349" s="180" t="n"/>
@@ -24295,20 +24391,627 @@
       <c r="Y349" s="180" t="n"/>
       <c r="Z349" s="180" t="n"/>
     </row>
+    <row r="350">
+      <c r="A350" s="205" t="inlineStr">
+        <is>
+          <t>6.71.1</t>
+        </is>
+      </c>
+      <c r="B350" s="206" t="inlineStr">
+        <is>
+          <t>Демонтаж воздуховода прямоугольного 300x250, изолированного</t>
+        </is>
+      </c>
+      <c r="C350" s="205" t="inlineStr">
+        <is>
+          <t>м.п.</t>
+        </is>
+      </c>
+      <c r="J350" s="205" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="K350" s="207" t="n">
+        <v>1140</v>
+      </c>
+      <c r="L350" s="207">
+        <f>J350*K350</f>
+        <v/>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="205" t="inlineStr">
+        <is>
+          <t>6.71.2</t>
+        </is>
+      </c>
+      <c r="B351" s="206" t="inlineStr">
+        <is>
+          <t>Демонтаж воздуховода прямоугольного 300x250, без изоляции</t>
+        </is>
+      </c>
+      <c r="C351" s="205" t="inlineStr">
+        <is>
+          <t>м.п.</t>
+        </is>
+      </c>
+      <c r="J351" s="205" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="K351" s="207" t="n">
+        <v>860</v>
+      </c>
+      <c r="L351" s="207">
+        <f>J351*K351</f>
+        <v/>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="205" t="inlineStr">
+        <is>
+          <t>6.71.3</t>
+        </is>
+      </c>
+      <c r="B352" s="206" t="inlineStr">
+        <is>
+          <t>Демонтаж воздуховода прямоугольного 400x200, изолированного</t>
+        </is>
+      </c>
+      <c r="C352" s="205" t="inlineStr">
+        <is>
+          <t>м.п.</t>
+        </is>
+      </c>
+      <c r="J352" s="205" t="n">
+        <v>17</v>
+      </c>
+      <c r="K352" s="207" t="n">
+        <v>1140</v>
+      </c>
+      <c r="L352" s="207">
+        <f>J352*K352</f>
+        <v/>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="205" t="inlineStr">
+        <is>
+          <t>6.71.4</t>
+        </is>
+      </c>
+      <c r="B353" s="206" t="inlineStr">
+        <is>
+          <t>Демонтаж воздуховода прямоугольного 400x200, без изоляции</t>
+        </is>
+      </c>
+      <c r="C353" s="205" t="inlineStr">
+        <is>
+          <t>м.п.</t>
+        </is>
+      </c>
+      <c r="J353" s="205" t="n">
+        <v>39.6</v>
+      </c>
+      <c r="K353" s="207" t="n">
+        <v>860</v>
+      </c>
+      <c r="L353" s="207">
+        <f>J353*K353</f>
+        <v/>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="205" t="inlineStr">
+        <is>
+          <t>6.71.5</t>
+        </is>
+      </c>
+      <c r="B354" s="206" t="inlineStr">
+        <is>
+          <t>Демонтаж воздуховода прямоугольного 500x250, изолированного</t>
+        </is>
+      </c>
+      <c r="C354" s="205" t="inlineStr">
+        <is>
+          <t>м.п.</t>
+        </is>
+      </c>
+      <c r="J354" s="205" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="K354" s="207" t="n">
+        <v>1360</v>
+      </c>
+      <c r="L354" s="207">
+        <f>J354*K354</f>
+        <v/>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="205" t="inlineStr">
+        <is>
+          <t>6.71.6</t>
+        </is>
+      </c>
+      <c r="B355" s="206" t="inlineStr">
+        <is>
+          <t>Демонтаж воздуховода прямоугольного 500x250, без изоляции</t>
+        </is>
+      </c>
+      <c r="C355" s="205" t="inlineStr">
+        <is>
+          <t>м.п.</t>
+        </is>
+      </c>
+      <c r="J355" s="205" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="K355" s="207" t="n">
+        <v>1040</v>
+      </c>
+      <c r="L355" s="207">
+        <f>J355*K355</f>
+        <v/>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="205" t="inlineStr">
+        <is>
+          <t>6.71.7</t>
+        </is>
+      </c>
+      <c r="B356" s="206" t="inlineStr">
+        <is>
+          <t>Демонтаж воздуховода прямоугольного 600x250, изолированного</t>
+        </is>
+      </c>
+      <c r="C356" s="205" t="inlineStr">
+        <is>
+          <t>м.п.</t>
+        </is>
+      </c>
+      <c r="J356" s="205" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="K356" s="207" t="n">
+        <v>1500</v>
+      </c>
+      <c r="L356" s="207">
+        <f>J356*K356</f>
+        <v/>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="205" t="inlineStr">
+        <is>
+          <t>6.71.8</t>
+        </is>
+      </c>
+      <c r="B357" s="206" t="inlineStr">
+        <is>
+          <t>Демонтаж воздуховода прямоугольного 600x250, без изоляции</t>
+        </is>
+      </c>
+      <c r="C357" s="205" t="inlineStr">
+        <is>
+          <t>м.п.</t>
+        </is>
+      </c>
+      <c r="J357" s="205" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="K357" s="207" t="n">
+        <v>1140</v>
+      </c>
+      <c r="L357" s="207">
+        <f>J357*K357</f>
+        <v/>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="205" t="inlineStr">
+        <is>
+          <t>6.71.9</t>
+        </is>
+      </c>
+      <c r="B358" s="206" t="inlineStr">
+        <is>
+          <t>Демонтаж воздуховода круглого Ø100, изолированного</t>
+        </is>
+      </c>
+      <c r="C358" s="205" t="inlineStr">
+        <is>
+          <t>м.п.</t>
+        </is>
+      </c>
+      <c r="J358" s="205" t="n">
+        <v>8</v>
+      </c>
+      <c r="K358" s="207" t="n">
+        <v>645</v>
+      </c>
+      <c r="L358" s="207">
+        <f>J358*K358</f>
+        <v/>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="205" t="inlineStr">
+        <is>
+          <t>6.71.10</t>
+        </is>
+      </c>
+      <c r="B359" s="206" t="inlineStr">
+        <is>
+          <t>Демонтаж воздуховода круглого Ø100, без изоляции</t>
+        </is>
+      </c>
+      <c r="C359" s="205" t="inlineStr">
+        <is>
+          <t>м.п.</t>
+        </is>
+      </c>
+      <c r="J359" s="205" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="K359" s="207" t="n">
+        <v>465</v>
+      </c>
+      <c r="L359" s="207">
+        <f>J359*K359</f>
+        <v/>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="205" t="inlineStr">
+        <is>
+          <t>6.71.11</t>
+        </is>
+      </c>
+      <c r="B360" s="206" t="inlineStr">
+        <is>
+          <t>Демонтаж воздуховода круглого Ø125, изолированного</t>
+        </is>
+      </c>
+      <c r="C360" s="205" t="inlineStr">
+        <is>
+          <t>м.п.</t>
+        </is>
+      </c>
+      <c r="J360" s="205" t="n">
+        <v>8</v>
+      </c>
+      <c r="K360" s="207" t="n">
+        <v>680</v>
+      </c>
+      <c r="L360" s="207">
+        <f>J360*K360</f>
+        <v/>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="205" t="inlineStr">
+        <is>
+          <t>6.71.12</t>
+        </is>
+      </c>
+      <c r="B361" s="206" t="inlineStr">
+        <is>
+          <t>Демонтаж воздуховода круглого Ø125, без изоляции</t>
+        </is>
+      </c>
+      <c r="C361" s="205" t="inlineStr">
+        <is>
+          <t>м.п.</t>
+        </is>
+      </c>
+      <c r="J361" s="205" t="n">
+        <v>2</v>
+      </c>
+      <c r="K361" s="207" t="n">
+        <v>500</v>
+      </c>
+      <c r="L361" s="207">
+        <f>J361*K361</f>
+        <v/>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="205" t="inlineStr">
+        <is>
+          <t>6.71.13</t>
+        </is>
+      </c>
+      <c r="B362" s="206" t="inlineStr">
+        <is>
+          <t>Демонтаж воздуховода круглого Ø200, изолированного (с КВК)</t>
+        </is>
+      </c>
+      <c r="C362" s="205" t="inlineStr">
+        <is>
+          <t>м.п.</t>
+        </is>
+      </c>
+      <c r="J362" s="205" t="n">
+        <v>70.3</v>
+      </c>
+      <c r="K362" s="207" t="n">
+        <v>785</v>
+      </c>
+      <c r="L362" s="207">
+        <f>J362*K362</f>
+        <v/>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="205" t="inlineStr">
+        <is>
+          <t>6.71.14</t>
+        </is>
+      </c>
+      <c r="B363" s="206" t="inlineStr">
+        <is>
+          <t>Демонтаж воздуховода круглого Ø200, без изоляции (с КВК)</t>
+        </is>
+      </c>
+      <c r="C363" s="205" t="inlineStr">
+        <is>
+          <t>м.п.</t>
+        </is>
+      </c>
+      <c r="J363" s="205" t="n">
+        <v>77.59999999999999</v>
+      </c>
+      <c r="K363" s="207" t="n">
+        <v>605</v>
+      </c>
+      <c r="L363" s="207">
+        <f>J363*K363</f>
+        <v/>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="205" t="inlineStr">
+        <is>
+          <t>6.71.15</t>
+        </is>
+      </c>
+      <c r="B364" s="206" t="inlineStr">
+        <is>
+          <t>Демонтаж воздуховода круглого Ø250, изолированного</t>
+        </is>
+      </c>
+      <c r="C364" s="205" t="inlineStr">
+        <is>
+          <t>м.п.</t>
+        </is>
+      </c>
+      <c r="J364" s="205" t="n">
+        <v>3</v>
+      </c>
+      <c r="K364" s="207" t="n">
+        <v>895</v>
+      </c>
+      <c r="L364" s="207">
+        <f>J364*K364</f>
+        <v/>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="205" t="inlineStr">
+        <is>
+          <t>6.71.16</t>
+        </is>
+      </c>
+      <c r="B365" s="206" t="inlineStr">
+        <is>
+          <t>Демонтаж воздуховода круглого Ø250, без изоляции</t>
+        </is>
+      </c>
+      <c r="C365" s="205" t="inlineStr">
+        <is>
+          <t>м.п.</t>
+        </is>
+      </c>
+      <c r="J365" s="205" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="K365" s="207" t="n">
+        <v>680</v>
+      </c>
+      <c r="L365" s="207">
+        <f>J365*K365</f>
+        <v/>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="205" t="inlineStr">
+        <is>
+          <t>6.71.17</t>
+        </is>
+      </c>
+      <c r="B366" s="206" t="inlineStr">
+        <is>
+          <t>Обрезка шпилек</t>
+        </is>
+      </c>
+      <c r="C366" s="205" t="inlineStr">
+        <is>
+          <t>шт.</t>
+        </is>
+      </c>
+      <c r="J366" s="205" t="n">
+        <v>348</v>
+      </c>
+      <c r="K366" s="207" t="n">
+        <v>105</v>
+      </c>
+      <c r="L366" s="207">
+        <f>J366*K366</f>
+        <v/>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="205" t="inlineStr">
+        <is>
+          <t>6.71.18</t>
+        </is>
+      </c>
+      <c r="B367" s="206" t="inlineStr">
+        <is>
+          <t>Демонтаж кронштейнов</t>
+        </is>
+      </c>
+      <c r="C367" s="205" t="inlineStr">
+        <is>
+          <t>шт.</t>
+        </is>
+      </c>
+      <c r="J367" s="205" t="n">
+        <v>188</v>
+      </c>
+      <c r="K367" s="207" t="n">
+        <v>250</v>
+      </c>
+      <c r="L367" s="207">
+        <f>J367*K367</f>
+        <v/>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="205" t="inlineStr">
+        <is>
+          <t>6.71.19</t>
+        </is>
+      </c>
+      <c r="B368" s="206" t="inlineStr">
+        <is>
+          <t>Герметизация отверстий воздуховодов</t>
+        </is>
+      </c>
+      <c r="C368" s="205" t="inlineStr">
+        <is>
+          <t>шт.</t>
+        </is>
+      </c>
+      <c r="J368" s="205" t="n">
+        <v>76</v>
+      </c>
+      <c r="K368" s="207" t="n">
+        <v>320</v>
+      </c>
+      <c r="L368" s="207">
+        <f>J368*K368</f>
+        <v/>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="205" t="inlineStr">
+        <is>
+          <t>6.71.20</t>
+        </is>
+      </c>
+      <c r="B369" s="206" t="inlineStr">
+        <is>
+          <t>Демонтаж проходок (обрезка ГКЛ, выемка из межстенового пространства)</t>
+        </is>
+      </c>
+      <c r="C369" s="205" t="inlineStr">
+        <is>
+          <t>шт.</t>
+        </is>
+      </c>
+      <c r="J369" s="205" t="n">
+        <v>50</v>
+      </c>
+      <c r="K369" s="207" t="n">
+        <v>860</v>
+      </c>
+      <c r="L369" s="207">
+        <f>J369*K369</f>
+        <v/>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="205" t="inlineStr">
+        <is>
+          <t>6.71.21</t>
+        </is>
+      </c>
+      <c r="B370" s="206" t="inlineStr">
+        <is>
+          <t>Подрезка и фиксация существующей изоляции на стыке с новой системой ОВ</t>
+        </is>
+      </c>
+      <c r="C370" s="205" t="inlineStr">
+        <is>
+          <t>м.п.</t>
+        </is>
+      </c>
+      <c r="J370" s="205" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="K370" s="207" t="n">
+        <v>430</v>
+      </c>
+      <c r="L370" s="207">
+        <f>J370*K370</f>
+        <v/>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="205" t="inlineStr">
+        <is>
+          <t>6.71.22</t>
+        </is>
+      </c>
+      <c r="B371" s="206" t="inlineStr">
+        <is>
+          <t>Сбор и перенос демонтированного к месту временного складирования</t>
+        </is>
+      </c>
+      <c r="C371" s="205" t="inlineStr">
+        <is>
+          <t>т</t>
+        </is>
+      </c>
+      <c r="J371" s="205" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="K371" s="207" t="n">
+        <v>8580</v>
+      </c>
+      <c r="L371" s="207">
+        <f>J371*K371</f>
+        <v/>
+      </c>
+    </row>
+    <row r="372">
+      <c r="B372" s="158" t="inlineStr">
+        <is>
+          <t>Итого по п. 6.71</t>
+        </is>
+      </c>
+      <c r="L372" s="208">
+        <f>SUM(L350:L371)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A3:X327"/>
-  <mergeCells count="11">
+  <mergeCells count="13">
     <mergeCell ref="S343:T343"/>
     <mergeCell ref="A329:K329"/>
     <mergeCell ref="S342:T342"/>
+    <mergeCell ref="S345:T345"/>
     <mergeCell ref="A332:L332"/>
     <mergeCell ref="R1:U1"/>
-    <mergeCell ref="S345:T345"/>
     <mergeCell ref="S2:W2"/>
+    <mergeCell ref="S346:T346"/>
+    <mergeCell ref="A348:L348"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="S344:T344"/>
+    <mergeCell ref="M1:Q1"/>
     <mergeCell ref="V1:X1"/>
-    <mergeCell ref="M1:Q1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>